<commit_message>
Sync QC views and add the world-history reading map.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/叶节点.xlsx
+++ b/叶节点.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\AppData\Local\Kingsoft\WPS Office\12.1.0.28022\office6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\worldForMe\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255"/>
+    <workbookView windowWidth="19440" windowHeight="12240"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
   <si>
     <t>叶</t>
   </si>
@@ -40,6 +40,9 @@
     <t>名称</t>
   </si>
   <si>
+    <t>是否已有</t>
+  </si>
+  <si>
     <t>T0</t>
   </si>
   <si>
@@ -220,54 +223,6 @@
     <t>历史叙事</t>
   </si>
   <si>
-    <t>QT8.1</t>
-  </si>
-  <si>
-    <t>武侠</t>
-  </si>
-  <si>
-    <t>QT8.2</t>
-  </si>
-  <si>
-    <t>欧洲骑士</t>
-  </si>
-  <si>
-    <t>QT8.3</t>
-  </si>
-  <si>
-    <t>日本武士与剑豪</t>
-  </si>
-  <si>
-    <t>QT8.4</t>
-  </si>
-  <si>
-    <t>欧洲剑客</t>
-  </si>
-  <si>
-    <t>QT8.5</t>
-  </si>
-  <si>
-    <t>西部</t>
-  </si>
-  <si>
-    <t>QT8.6</t>
-  </si>
-  <si>
-    <t>Gaucho</t>
-  </si>
-  <si>
-    <t>QT8.7</t>
-  </si>
-  <si>
-    <t>侠盗</t>
-  </si>
-  <si>
-    <t>QT8.8</t>
-  </si>
-  <si>
-    <t>海盗</t>
-  </si>
-  <si>
     <t>QT9</t>
   </si>
   <si>
@@ -434,6 +389,168 @@
   </si>
   <si>
     <t>信仰、伦理与超越</t>
+  </si>
+  <si>
+    <t>QX</t>
+  </si>
+  <si>
+    <t>文学意象与场景</t>
+  </si>
+  <si>
+    <t>QC1.1.1</t>
+  </si>
+  <si>
+    <t>QC1.1.2</t>
+  </si>
+  <si>
+    <t>QC1.1.3</t>
+  </si>
+  <si>
+    <t>QC1.1.4</t>
+  </si>
+  <si>
+    <t>QC1.1.5</t>
+  </si>
+  <si>
+    <t>QC1.1.6</t>
+  </si>
+  <si>
+    <t>QC1.1.7</t>
+  </si>
+  <si>
+    <t>QC1.1.8</t>
+  </si>
+  <si>
+    <t>QC1.1.9</t>
+  </si>
+  <si>
+    <t>QC1.1.10</t>
+  </si>
+  <si>
+    <t>QC1.1.11</t>
+  </si>
+  <si>
+    <t>QC1.2.1</t>
+  </si>
+  <si>
+    <t>QC1.2.2</t>
+  </si>
+  <si>
+    <t>QC1.2.3</t>
+  </si>
+  <si>
+    <t>QC1.2.4</t>
+  </si>
+  <si>
+    <t>QC1.2.5</t>
+  </si>
+  <si>
+    <t>QC1.2.6</t>
+  </si>
+  <si>
+    <t>QC1.2.7</t>
+  </si>
+  <si>
+    <t>QC1.2.8</t>
+  </si>
+  <si>
+    <t>QC1.2.9</t>
+  </si>
+  <si>
+    <t>QC1.2.10</t>
+  </si>
+  <si>
+    <t>QC1.2.11</t>
+  </si>
+  <si>
+    <t>QC1.2.12</t>
+  </si>
+  <si>
+    <t>QC1.2.13</t>
+  </si>
+  <si>
+    <t>QC1.2.14</t>
+  </si>
+  <si>
+    <t>QC1.2.15</t>
+  </si>
+  <si>
+    <t>QC1.2.16</t>
+  </si>
+  <si>
+    <t>QC1.2.17</t>
+  </si>
+  <si>
+    <t>QC1.2.18</t>
+  </si>
+  <si>
+    <t>QC1.2.19</t>
+  </si>
+  <si>
+    <t>QC1.2.20</t>
+  </si>
+  <si>
+    <t>QC2.1</t>
+  </si>
+  <si>
+    <t>QC2.2</t>
+  </si>
+  <si>
+    <t>QC2.3</t>
+  </si>
+  <si>
+    <t>QC2.4</t>
+  </si>
+  <si>
+    <t>QC2.5</t>
+  </si>
+  <si>
+    <t>QC2.6</t>
+  </si>
+  <si>
+    <t>QC2.7</t>
+  </si>
+  <si>
+    <t>QC2.8</t>
+  </si>
+  <si>
+    <t>QC2.9</t>
+  </si>
+  <si>
+    <t>QC2.10</t>
+  </si>
+  <si>
+    <t>QC2.11</t>
+  </si>
+  <si>
+    <t>QC2.12</t>
+  </si>
+  <si>
+    <t>QC2.13</t>
+  </si>
+  <si>
+    <t>QC2.14</t>
+  </si>
+  <si>
+    <t>QC2.15</t>
+  </si>
+  <si>
+    <t>QC2.16</t>
+  </si>
+  <si>
+    <t>QC2.17</t>
+  </si>
+  <si>
+    <t>QC2.18</t>
+  </si>
+  <si>
+    <t>QC2.19</t>
+  </si>
+  <si>
+    <t>QC2.20</t>
+  </si>
+  <si>
+    <t>QC3</t>
   </si>
 </sst>
 </file>
@@ -446,26 +563,13 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF333333"/>
-      <name val="Helvetica"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF333333"/>
-      <name val="Helvetica"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -612,7 +716,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -621,18 +725,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F8F8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -818,40 +910,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFDFE2E5"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFDFE2E5"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFDFE2E5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFDFE2E5"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFDFE2E5"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFDFE2E5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFDFE2E5"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -972,52 +1036,58 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1029,90 +1099,75 @@
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1640,543 +1695,861 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <dimension ref="A1:C112"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
+  <cols>
+    <col min="2" max="2" width="34.375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="16.5" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" ht="15.75" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" ht="15.75" spans="1:2">
-      <c r="A4" s="2" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="15.75" spans="1:2">
-      <c r="A5" s="3" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="15.75" spans="1:2">
-      <c r="A6" s="2" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" ht="15.75" spans="1:2">
-      <c r="A7" s="3" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" ht="15.75" spans="1:2">
-      <c r="A8" s="2" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" ht="15.75" spans="1:2">
-      <c r="A9" s="2" t="s">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" ht="15.75" spans="1:2">
-      <c r="A10" s="3" t="s">
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" ht="15.75" spans="1:2">
-      <c r="A11" s="2" t="s">
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" ht="15.75" spans="1:2">
-      <c r="A12" s="3" t="s">
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" ht="15.75" spans="1:2">
-      <c r="A13" s="2" t="s">
+      <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" ht="15.75" spans="1:2">
-      <c r="A14" s="3" t="s">
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" ht="15.75" spans="1:2">
-      <c r="A15" s="2" t="s">
+      <c r="B14" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" ht="15.75" spans="1:2">
-      <c r="A16" s="3" t="s">
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" ht="15.75" spans="1:2">
-      <c r="A17" s="2" t="s">
+      <c r="B16" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" ht="15.75" spans="1:2">
-      <c r="A18" s="2" t="s">
+      <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" ht="15.75" spans="1:2">
-      <c r="A19" s="2" t="s">
+      <c r="B18" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" ht="15.75" spans="1:2">
-      <c r="A20" s="3" t="s">
+      <c r="B19" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" ht="15.75" spans="1:2">
-      <c r="A21" s="2" t="s">
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="22" ht="15.75" spans="1:2">
-      <c r="A22" s="3" t="s">
+      <c r="B21" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" ht="15.75" spans="1:2">
-      <c r="A23" s="2" t="s">
+      <c r="B22" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="24" ht="15.75" spans="1:2">
-      <c r="A24" s="3" t="s">
+      <c r="B23" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" ht="15.75" spans="1:2">
-      <c r="A25" s="2" t="s">
+      <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" ht="15.75" spans="1:2">
-      <c r="A26" s="3" t="s">
+      <c r="B25" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="3" t="s">
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="27" ht="15.75" spans="1:2">
-      <c r="A27" s="2" t="s">
+      <c r="B26" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="2" t="s">
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" ht="15.75" spans="1:2">
-      <c r="A28" s="3" t="s">
+      <c r="B27" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="3" t="s">
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" ht="15.75" spans="1:2">
-      <c r="A29" s="2" t="s">
+      <c r="B28" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="2" t="s">
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" ht="15.75" spans="1:2">
-      <c r="A30" s="3" t="s">
+      <c r="B29" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="3" t="s">
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="31" ht="15.75" spans="1:2">
-      <c r="A31" s="2" t="s">
+      <c r="B30" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="2" t="s">
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="32" ht="15.75" spans="1:2">
-      <c r="A32" s="3" t="s">
+      <c r="B31" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="3" t="s">
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="33" ht="15.75" spans="1:2">
-      <c r="A33" s="2" t="s">
+      <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="34" ht="15.75" spans="1:2">
-      <c r="A34" s="3" t="s">
+      <c r="B33" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="3" t="s">
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="35" ht="15.75" spans="1:2">
-      <c r="A35" s="2" t="s">
+      <c r="B34" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="2" t="s">
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="36" ht="15.75" spans="1:2">
-      <c r="A36" s="3" t="s">
+      <c r="B35" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="3" t="s">
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="37" ht="15.75" spans="1:2">
-      <c r="A37" s="2" t="s">
+      <c r="B36" t="s">
         <v>72</v>
       </c>
-      <c r="B37" s="2" t="s">
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="38" ht="15.75" spans="1:2">
-      <c r="A38" s="3" t="s">
+      <c r="B37" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="3" t="s">
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="39" ht="15.75" spans="1:2">
-      <c r="A39" s="2" t="s">
+      <c r="B38" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="40" ht="15.75" spans="1:2">
-      <c r="A40" s="3" t="s">
+      <c r="B39" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="C39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="41" ht="15.75" spans="1:2">
-      <c r="A41" s="2" t="s">
+      <c r="B40" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="42" ht="15.75" spans="1:2">
-      <c r="A42" s="3" t="s">
+      <c r="B41" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="C41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="43" ht="15.75" spans="1:2">
-      <c r="A43" s="2" t="s">
+      <c r="B42" t="s">
         <v>84</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="44" ht="15.75" spans="1:2">
-      <c r="A44" s="3" t="s">
+      <c r="B43" t="s">
         <v>86</v>
       </c>
-      <c r="B44" s="3" t="s">
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="45" ht="15.75" spans="1:2">
-      <c r="A45" s="2" t="s">
+      <c r="B44" t="s">
         <v>88</v>
       </c>
-      <c r="B45" s="2" t="s">
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="46" ht="15.75" spans="1:2">
-      <c r="A46" s="2" t="s">
+      <c r="B45" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="2" t="s">
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="47" ht="15.75" spans="1:2">
-      <c r="A47" s="3" t="s">
+      <c r="B46" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="3" t="s">
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="48" ht="15.75" spans="1:2">
-      <c r="A48" s="2" t="s">
+      <c r="B47" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="2" t="s">
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="49" ht="15.75" spans="1:2">
-      <c r="A49" s="3" t="s">
+      <c r="B48" t="s">
         <v>96</v>
       </c>
-      <c r="B49" s="3" t="s">
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="50" ht="15.75" spans="1:2">
-      <c r="A50" s="2" t="s">
+      <c r="B49" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="2" t="s">
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="51" ht="15.75" spans="1:2">
-      <c r="A51" s="3" t="s">
+      <c r="B50" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="3" t="s">
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="52" ht="15.75" spans="1:2">
-      <c r="A52" s="2" t="s">
+      <c r="B51" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="2" t="s">
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53" ht="15.75" spans="1:2">
-      <c r="A53" s="3" t="s">
+      <c r="B52" t="s">
         <v>104</v>
       </c>
-      <c r="B53" s="3" t="s">
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="54" ht="15.75" spans="1:2">
-      <c r="A54" s="2" t="s">
+      <c r="B53" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="2" t="s">
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="55" ht="15.75" spans="1:2">
-      <c r="A55" s="3" t="s">
+      <c r="B54" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="3" t="s">
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="56" ht="15.75" spans="1:2">
-      <c r="A56" s="2" t="s">
+      <c r="B55" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="2" t="s">
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="57" ht="15.75" spans="1:2">
-      <c r="A57" s="3" t="s">
+      <c r="B56" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="3" t="s">
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="58" ht="15.75" spans="1:2">
-      <c r="A58" s="2" t="s">
+      <c r="B57" t="s">
         <v>114</v>
       </c>
-      <c r="B58" s="2" t="s">
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="59" ht="15.75" spans="1:2">
-      <c r="A59" s="3" t="s">
+      <c r="B58" t="s">
         <v>116</v>
       </c>
-      <c r="B59" s="3" t="s">
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="60" ht="15.75" spans="1:2">
-      <c r="A60" s="2" t="s">
+      <c r="B59" t="s">
         <v>118</v>
       </c>
-      <c r="B60" s="2" t="s">
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="61" ht="15.75" spans="1:2">
-      <c r="A61" s="3" t="s">
+      <c r="B60" t="s">
         <v>120</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="C60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="62" ht="15.75" spans="1:2">
-      <c r="A62" s="2" t="s">
+      <c r="C61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
         <v>122</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="C62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="A63" t="s">
+      <c r="C63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
         <v>124</v>
       </c>
-      <c r="B63" t="s">
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
-      <c r="A64" t="s">
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
         <v>126</v>
       </c>
-      <c r="B64" t="s">
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
-      <c r="A65" t="s">
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
         <v>128</v>
       </c>
-      <c r="B65" t="s">
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
-      <c r="A66" t="s">
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>130</v>
       </c>
-      <c r="B66" t="s">
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
-      <c r="A67" t="s">
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
         <v>132</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
         <v>133</v>
+      </c>
+      <c r="C73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>135</v>
+      </c>
+      <c r="C75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>